<commit_message>
Updated files for 4.0.4
</commit_message>
<xml_diff>
--- a/InputData/elec/BSfGBP/BAU Subsidy for Grid Battery Production.xlsx
+++ b/InputData/elec/BSfGBP/BAU Subsidy for Grid Battery Production.xlsx
@@ -1,24 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28816"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\elec\BSfGBP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BSfGBP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C593B89-7C5B-422D-AEFA-1E1F48F5216D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{DE830CDA-2171-4933-BA48-7F50760EB19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75EC6EC5-DA5A-4AAB-BA6E-68F346BD555F}"/>
   <bookViews>
-    <workbookView xWindow="31935" yWindow="3675" windowWidth="19200" windowHeight="11205" activeTab="2" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="2" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Phase Out" sheetId="3" r:id="rId2"/>
     <sheet name="BSfGBP" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -35,52 +38,46 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>BSfVBP BAU Subsidy for Vehicle Battery Production</t>
+  </si>
   <si>
     <t>Sources:</t>
   </si>
   <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>File is mainly to help reflect US IRA data. Data can be 0'd out here.</t>
+  </si>
+  <si>
+    <t>In the US, the Inflation Reduction Act includes a credit of $35/kWh for battery cells and $10/kWh for assembly for grid</t>
+  </si>
+  <si>
+    <t>batteries. This value is not inflation adjusted.</t>
+  </si>
+  <si>
+    <t>2023 to 2012 USD</t>
+  </si>
+  <si>
+    <t>2024 to 2012 USD</t>
+  </si>
+  <si>
+    <t>annual inflation assumption after 2024</t>
+  </si>
+  <si>
+    <t>$/MWh</t>
+  </si>
+  <si>
     <t>Price</t>
-  </si>
-  <si>
-    <t>Notes:</t>
-  </si>
-  <si>
-    <t>BSfVBP BAU Subsidy for Vehicle Battery Production</t>
-  </si>
-  <si>
-    <t>United States Congress</t>
-  </si>
-  <si>
-    <t>H.R. 5376 - Inflation Reduction Act of 2022</t>
-  </si>
-  <si>
-    <t>https://www.congress.gov/bill/117th-congress/house-bill/5376/text</t>
-  </si>
-  <si>
-    <t>2023 to 2012 USD</t>
-  </si>
-  <si>
-    <t>2024 to 2012 USD</t>
-  </si>
-  <si>
-    <t>annual inflation assumption after 2024</t>
-  </si>
-  <si>
-    <t>batteries. This value is not inflation adjusted.</t>
-  </si>
-  <si>
-    <t>$/MWh</t>
-  </si>
-  <si>
-    <t>In the US, the Inflation Reduction Act includes a credit of $35/kWh for battery cells and $10/kWh for assembly for grid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,13 +122,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -151,9 +149,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -191,7 +189,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -297,7 +295,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -439,7 +437,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -447,77 +445,70 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF982137-6F01-4109-8226-D4C6F3731BA9}">
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="101.26953125" customWidth="1"/>
+    <col min="2" max="2" width="101.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B4" s="2">
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B5" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="B4" s="2"/>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="B5" s="2"/>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2">
+      <c r="A9" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13">
         <v>0.75350342301658668</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14">
+        <v>0.73</v>
+      </c>
+      <c r="B14" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13">
-        <v>0.73</v>
-      </c>
-      <c r="B13" t="s">
+    <row r="15" spans="1:2">
+      <c r="A15" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="B15" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="3">
-        <v>0.03</v>
-      </c>
-      <c r="B14" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -528,9 +519,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B33CFD9F-5CAA-490F-A0C6-0C0A5236B09C}">
   <dimension ref="B2:K3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:11">
       <c r="B2">
         <v>2023</v>
       </c>
@@ -562,7 +553,7 @@
         <v>2032</v>
       </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:11">
       <c r="B3">
         <v>1</v>
       </c>
@@ -604,113 +595,110 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AE2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.54296875" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="E1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="H1">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="I1">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="J1">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="K1">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="L1">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="M1">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="N1">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="O1">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="P1">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="Q1">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="R1">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="S1">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="T1">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="U1">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="V1">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="W1">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="X1">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="Y1">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="Z1">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="AA1">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="AB1">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="AC1">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="AD1">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AE1">
-        <v>2049</v>
-      </c>
-      <c r="AF1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -722,44 +710,34 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <f>45*About!$A$12*10^3</f>
-        <v>33907.654035746404</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <f>45*About!$A$13*10^3</f>
-        <v>32850</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <f>$F2*(1-About!$A$14)^(G1-$F1)*'Phase Out'!D3</f>
-        <v>31864.5</v>
+        <v>0</v>
       </c>
       <c r="H2">
-        <f>$F2*(1-About!$A$14)^(H1-$F1)*'Phase Out'!E3</f>
-        <v>30908.564999999999</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <f>$F2*(1-About!$A$14)^(I1-$F1)*'Phase Out'!F3</f>
-        <v>29981.30805</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <f>$F2*(1-About!$A$14)^(J1-$F1)*'Phase Out'!G3</f>
-        <v>29081.868808499999</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <f>$F2*(1-About!$A$14)^(K1-$F1)*'Phase Out'!H3</f>
-        <v>28209.412744244997</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <f>$F2*(1-About!$A$14)^(L1-$F1)*'Phase Out'!I3</f>
-        <v>20522.347771438235</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <f>$F2*(1-About!$A$14)^(M1-$F1)*'Phase Out'!J3</f>
-        <v>13271.118225530059</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <f>$F2*(1-About!$A$14)^(N1-$F1)*'Phase Out'!K3</f>
-        <v>6436.4923393820782</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -810,13 +788,181 @@
         <v>0</v>
       </c>
       <c r="AE2">
-        <v>0</v>
-      </c>
-      <c r="AF2">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002041A8AB53924247A2770D65450F5227" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="90fff4f083191fe75a03dbd50c7739fc">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1659011e-6b88-4225-9a61-aaf33aaf19e8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7fee88694a371868130ae0617c69143c" ns2:_="">
+    <xsd:import namespace="1659011e-6b88-4225-9a61-aaf33aaf19e8"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="1659011e-6b88-4225-9a61-aaf33aaf19e8" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04CDCC88-E755-4C08-8FC2-EFA95D88AB39}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBF01092-65CD-4846-84A4-8BA5E7F3DE75}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D3F6B8D-C427-451A-A517-E363B6FDCC24}"/>
 </file>
</xml_diff>

<commit_message>
updating time series for BSfGBP, FoGBPD, and ACTR
</commit_message>
<xml_diff>
--- a/InputData/elec/BSfGBP/BAU Subsidy for Grid Battery Production.xlsx
+++ b/InputData/elec/BSfGBP/BAU Subsidy for Grid Battery Production.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BSfGBP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\Indonesia EPS\InputData\elec\BSfGBP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{DE830CDA-2171-4933-BA48-7F50760EB19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75EC6EC5-DA5A-4AAB-BA6E-68F346BD555F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33095175-8ECC-4B2E-89A1-B31A7BB6CC35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="2" activeTab="2" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
+    <workbookView xWindow="38190" yWindow="1815" windowWidth="23235" windowHeight="13365" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,14 +122,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -149,9 +148,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -189,7 +188,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -295,7 +294,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -437,7 +436,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -446,48 +445,48 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF982137-6F01-4109-8226-D4C6F3731BA9}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="101.28515625" customWidth="1"/>
+    <col min="2" max="2" width="101.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" s="2"/>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>0.75350342301658668</v>
       </c>
@@ -495,7 +494,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>0.73</v>
       </c>
@@ -503,7 +502,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>0.03</v>
       </c>
@@ -519,9 +518,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B33CFD9F-5CAA-490F-A0C6-0C0A5236B09C}">
   <dimension ref="B2:K3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:11">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B2">
         <v>2023</v>
       </c>
@@ -553,7 +552,7 @@
         <v>2032</v>
       </c>
     </row>
-    <row r="3" spans="2:11">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>1</v>
       </c>
@@ -595,108 +594,111 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:AF2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="1" max="2" width="24.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
       <c r="B1">
+        <v>2020</v>
+      </c>
+      <c r="C1">
         <v>2021</v>
       </c>
-      <c r="C1">
+      <c r="D1">
         <v>2022</v>
       </c>
-      <c r="D1">
+      <c r="E1">
         <v>2023</v>
       </c>
-      <c r="E1">
+      <c r="F1">
         <v>2024</v>
       </c>
-      <c r="F1">
+      <c r="G1">
         <v>2025</v>
       </c>
-      <c r="G1">
+      <c r="H1">
         <v>2026</v>
       </c>
-      <c r="H1">
+      <c r="I1">
         <v>2027</v>
       </c>
-      <c r="I1">
+      <c r="J1">
         <v>2028</v>
       </c>
-      <c r="J1">
+      <c r="K1">
         <v>2029</v>
       </c>
-      <c r="K1">
+      <c r="L1">
         <v>2030</v>
       </c>
-      <c r="L1">
+      <c r="M1">
         <v>2031</v>
       </c>
-      <c r="M1">
+      <c r="N1">
         <v>2032</v>
       </c>
-      <c r="N1">
+      <c r="O1">
         <v>2033</v>
       </c>
-      <c r="O1">
+      <c r="P1">
         <v>2034</v>
       </c>
-      <c r="P1">
+      <c r="Q1">
         <v>2035</v>
       </c>
-      <c r="Q1">
+      <c r="R1">
         <v>2036</v>
       </c>
-      <c r="R1">
+      <c r="S1">
         <v>2037</v>
       </c>
-      <c r="S1">
+      <c r="T1">
         <v>2038</v>
       </c>
-      <c r="T1">
+      <c r="U1">
         <v>2039</v>
       </c>
-      <c r="U1">
+      <c r="V1">
         <v>2040</v>
       </c>
-      <c r="V1">
+      <c r="W1">
         <v>2041</v>
       </c>
-      <c r="W1">
+      <c r="X1">
         <v>2042</v>
       </c>
-      <c r="X1">
+      <c r="Y1">
         <v>2043</v>
       </c>
-      <c r="Y1">
+      <c r="Z1">
         <v>2044</v>
       </c>
-      <c r="Z1">
+      <c r="AA1">
         <v>2045</v>
       </c>
-      <c r="AA1">
+      <c r="AB1">
         <v>2046</v>
       </c>
-      <c r="AB1">
+      <c r="AC1">
         <v>2047</v>
       </c>
-      <c r="AC1">
+      <c r="AD1">
         <v>2048</v>
       </c>
-      <c r="AD1">
+      <c r="AE1">
         <v>2049</v>
       </c>
-      <c r="AE1">
+      <c r="AF1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -788,6 +790,9 @@
         <v>0</v>
       </c>
       <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
         <v>0</v>
       </c>
     </row>
@@ -797,21 +802,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002041A8AB53924247A2770D65450F5227" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="90fff4f083191fe75a03dbd50c7739fc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1659011e-6b88-4225-9a61-aaf33aaf19e8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7fee88694a371868130ae0617c69143c" ns2:_="">
     <xsd:import namespace="1659011e-6b88-4225-9a61-aaf33aaf19e8"/>
@@ -955,14 +945,52 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04CDCC88-E755-4C08-8FC2-EFA95D88AB39}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D3F6B8D-C427-451A-A517-E363B6FDCC24}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1659011e-6b88-4225-9a61-aaf33aaf19e8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBF01092-65CD-4846-84A4-8BA5E7F3DE75}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBF01092-65CD-4846-84A4-8BA5E7F3DE75}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D3F6B8D-C427-451A-A517-E363B6FDCC24}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04CDCC88-E755-4C08-8FC2-EFA95D88AB39}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>